<commit_message>
Bloque C1-1 (servidor): usuarios, sesión, bitácora, parámetros, motivos, catálogo y bodega
- Autenticación: bloqueo tras intentos fallidos, cambio de clave en el primer
  acceso, cierre de sesión por inactividad (parámetro de M-19) y acceso
  cerrado de inmediato al desactivar a un usuario.
- Bitácora inmutable: la base de datos rechaza UPDATE, DELETE y TRUNCATE, y
  cada registro encadena el hash del anterior; se detecta cualquier alteración.
- Usuarios y roles, parámetros con rango y registro anterior/nuevo, motivos
  tipificados, catálogo (referencias, tallas, colores, SKU) y estructura de
  bodega (zonas, ubicaciones, capacidad) con sus reglas.
- Pruebas contra una base de datos propia: 58 pasan, 3 pendientes (dependen
  del kardex del bloque C1-3).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/datos_ficticios.xlsx
+++ b/data/datos_ficticios.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="bodegas" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="zonas" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="ubicaciones" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="motivos" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="182">
   <si>
     <t>login</t>
   </si>
@@ -502,6 +503,66 @@
   </si>
   <si>
     <t>CUA-02</t>
+  </si>
+  <si>
+    <t>tipo_operacion</t>
+  </si>
+  <si>
+    <t>exige_evidencia</t>
+  </si>
+  <si>
+    <t>AJUSTE</t>
+  </si>
+  <si>
+    <t>Diferencia detectada en conteo</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Error de registro corregido</t>
+  </si>
+  <si>
+    <t>Mercancía dañada</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Mercancía perdida</t>
+  </si>
+  <si>
+    <t>ANULACION</t>
+  </si>
+  <si>
+    <t>Movimiento registrado por error</t>
+  </si>
+  <si>
+    <t>Cantidad mal digitada</t>
+  </si>
+  <si>
+    <t>SALIDA</t>
+  </si>
+  <si>
+    <t>Consumo en producción</t>
+  </si>
+  <si>
+    <t>Despacho</t>
+  </si>
+  <si>
+    <t>Devolución al origen</t>
+  </si>
+  <si>
+    <t>Baja por daño</t>
+  </si>
+  <si>
+    <t>DESCARTE_ALERTA</t>
+  </si>
+  <si>
+    <t>Alerta atendida</t>
+  </si>
+  <si>
+    <t>Falsa alarma</t>
   </si>
 </sst>
 </file>
@@ -1977,4 +2038,158 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B12" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>179</v>
+      </c>
+      <c r="B13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bloque C1-3: entradas, piezas y ubicación (HU-ENT-001/002/003/004/006/009)
Documento de entrada, recepción por piezas, comparación esperado/recibido, confirmación por segunda persona, kardex inmutable con existencia derivada y no negativa en la base de datos, y propuesta y confirmación de ubicación. Corrige el cliente web: los POST sin cuerpo (Salir, desactivar, cerrar recepción) fallaban con 400.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/datos_ficticios.xlsx
+++ b/data/datos_ficticios.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="183">
   <si>
     <t>login</t>
   </si>
@@ -371,6 +371,9 @@
   </si>
   <si>
     <t>RECEPCION</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>ALM-A</t>
@@ -1581,10 +1584,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>113</v>
       </c>
@@ -1597,8 +1600,11 @@
       <c r="D1" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>111</v>
       </c>
@@ -1611,75 +1617,93 @@
       <c r="D2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>111</v>
       </c>
       <c r="B3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" t="s">
         <v>118</v>
       </c>
-      <c r="C3" t="s">
-        <v>119</v>
-      </c>
-      <c r="D3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C4" t="s">
-        <v>122</v>
-      </c>
-      <c r="D4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D7" t="s">
-        <v>130</v>
+        <v>131</v>
+      </c>
+      <c r="E7" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1698,7 +1722,7 @@
         <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>25</v>
@@ -1712,7 +1736,7 @@
         <v>115</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1723,7 +1747,7 @@
         <v>115</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1734,7 +1758,7 @@
         <v>115</v>
       </c>
       <c r="C4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1742,10 +1766,10 @@
         <v>111</v>
       </c>
       <c r="B5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1753,10 +1777,10 @@
         <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1764,10 +1788,10 @@
         <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1775,10 +1799,10 @@
         <v>111</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1786,10 +1810,10 @@
         <v>111</v>
       </c>
       <c r="B9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1797,10 +1821,10 @@
         <v>111</v>
       </c>
       <c r="B10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1808,10 +1832,10 @@
         <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1819,10 +1843,10 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1830,10 +1854,10 @@
         <v>111</v>
       </c>
       <c r="B13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1841,10 +1865,10 @@
         <v>111</v>
       </c>
       <c r="B14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1852,10 +1876,10 @@
         <v>111</v>
       </c>
       <c r="B15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1863,10 +1887,10 @@
         <v>111</v>
       </c>
       <c r="B16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1874,10 +1898,10 @@
         <v>111</v>
       </c>
       <c r="B17" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1885,10 +1909,10 @@
         <v>111</v>
       </c>
       <c r="B18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1896,10 +1920,10 @@
         <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C19" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1907,10 +1931,10 @@
         <v>111</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C20" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1918,10 +1942,10 @@
         <v>111</v>
       </c>
       <c r="B21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C21" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1929,10 +1953,10 @@
         <v>111</v>
       </c>
       <c r="B22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1940,10 +1964,10 @@
         <v>111</v>
       </c>
       <c r="B23" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C23" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1951,10 +1975,10 @@
         <v>111</v>
       </c>
       <c r="B24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1962,10 +1986,10 @@
         <v>111</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1973,10 +1997,10 @@
         <v>111</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1984,10 +2008,10 @@
         <v>111</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1995,10 +2019,10 @@
         <v>111</v>
       </c>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -2006,10 +2030,10 @@
         <v>111</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C29" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -2017,10 +2041,10 @@
         <v>111</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C30" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2028,10 +2052,10 @@
         <v>111</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -2047,145 +2071,145 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3" t="s">
         <v>167</v>
-      </c>
-      <c r="C3" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" t="s">
         <v>170</v>
-      </c>
-      <c r="C5" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>